<commit_message>
fix: all fixes - font, permissions, labels, canView
</commit_message>
<xml_diff>
--- a/3TEST-template_import_khach_hang.xlsx
+++ b/3TEST-template_import_khach_hang.xlsx
@@ -15,12 +15,12 @@
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
   <si>
     <t>Tên KH</t>
   </si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -575,8 +578,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.796875" customWidth="1"/>
     <col min="2" max="2" width="15.796875" style="1" customWidth="1"/>
@@ -587,7 +590,7 @@
     <col min="8" max="9" width="14.796875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +619,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -644,8 +647,11 @@
       <c r="I2" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -674,7 +680,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -703,7 +709,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -732,7 +738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -761,7 +767,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -790,7 +796,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -819,7 +825,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -848,7 +854,6 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -861,13 +866,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14.796875" customWidth="1"/>
     <col min="3" max="3" width="65.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -878,7 +883,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -889,7 +894,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -900,7 +905,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -911,7 +916,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -922,7 +927,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -933,7 +938,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -944,7 +949,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -955,7 +960,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -966,7 +971,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>

</xml_diff>